<commit_message>
Record five owner Kashmiri corrections in Hadith vocabulary CSV, Excel and review ledger
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -123,12 +123,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">کانهه تقسیمہٕ نِش تراوُن</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G5" s="4">
@@ -174,12 +174,12 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">نارس منز بُتھ  کٕن تراونہ یُن</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G6" s="5">
@@ -225,12 +225,12 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">پننِس خانٛدارس ناشکرا</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G7" s="4">
@@ -378,12 +378,12 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">کٲنٛسہِ  بے عزتی کَرٕن  ماجہِ ہٕنٛز زریع</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G10" s="5">
@@ -429,12 +429,12 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">کٲنهه شَخصَس قَتل کَرنُک اِرادٕ تھاوُن</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G11" s="4">
@@ -3478,7 +3478,7 @@
   <autoFilter ref="A4:K70"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="F5:F70">
-      <formula1>"Needs review,Approved,Needs correction"</formula1>
+      <formula1>"Needs review,Approved,Needs correction,Owner corrected"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>

</xml_diff>

<commit_message>
Update Bukhari 27–100 XLSX with confirmed vocabulary corrections 11–20
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G15" s="4">
@@ -661,7 +661,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G16" s="5">
@@ -712,7 +712,7 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner-approved prepositional construction reused; guard duty translation is a fresh draft.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G17" s="4">
@@ -763,7 +763,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G18" s="5">
@@ -814,7 +814,7 @@
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G19" s="4">
@@ -865,7 +865,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G20" s="5">
@@ -916,7 +916,7 @@
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -939,12 +939,12 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">وٕشکہٕ / کٕنُک</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G21" s="4">
@@ -967,7 +967,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm both crop words with a native speaker.</t>
+          <t xml:space="preserve">Owner supplied exact Kashmiri words: barley وٕشکہٕ; wheat کٕنُک. Individual words owner corrected; full phrase draft.</t>
         </is>
       </c>
     </row>
@@ -990,12 +990,12 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">أکِس دۄہس تیوہارک پٲٹھۍ مانُن</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G22" s="5">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner supplied exact phrase on 2026-10-28.</t>
         </is>
       </c>
     </row>
@@ -1041,12 +1041,12 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مٔس — maes waekrith aaasun</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G23" s="4">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Natural Kashmiri idiom and spelling need checking.</t>
+          <t xml:space="preserve">Owner confirmed noun مٔس and romanized phrase maes waekrith aaasun; complete Perso-Arabic spelling not confirmed.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G24" s="5">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update owner-reviewed Kashmiri Bukhari vocabulary through item 20
* Accept Bukhari vocabulary 11–16 and 20; preserve owner corrections 17–19

* Document precise owner corrections for barley wheat festival and hair

* Extend owner vocabulary correction ledger through items 11–20

* Update Bukhari 27–100 XLSX with confirmed vocabulary corrections 11–20

* Reflect updated Excel workbook with owner vocabulary review through item 20
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G15" s="4">
@@ -661,7 +661,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G16" s="5">
@@ -712,7 +712,7 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner-approved prepositional construction reused; guard duty translation is a fresh draft.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G17" s="4">
@@ -763,7 +763,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G18" s="5">
@@ -814,7 +814,7 @@
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G19" s="4">
@@ -865,7 +865,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G20" s="5">
@@ -916,7 +916,7 @@
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -939,12 +939,12 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">وٕشکہٕ / کٕنُک</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G21" s="4">
@@ -967,7 +967,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm both crop words with a native speaker.</t>
+          <t xml:space="preserve">Owner supplied exact Kashmiri words: barley وٕشکہٕ; wheat کٕنُک. Individual words owner corrected; full phrase draft.</t>
         </is>
       </c>
     </row>
@@ -990,12 +990,12 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">أکِس دۄہس تیوہارک پٲٹھۍ مانُن</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G22" s="5">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner supplied exact phrase on 2026-10-28.</t>
         </is>
       </c>
     </row>
@@ -1041,12 +1041,12 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مٔس — maes waekrith aaasun</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G23" s="4">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Natural Kashmiri idiom and spelling need checking.</t>
+          <t xml:space="preserve">Owner confirmed noun مٔس and romanized phrase maes waekrith aaasun; complete Perso-Arabic spelling not confirmed.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G24" s="5">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previous draft wording on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Bukhari review Excel with owner wording and acceptances through item 30
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -1143,12 +1143,12 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">فِسق — گُناہگارٕ عمل</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G25" s="4">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">دۄن شَخصَن دَرمِیان جَھگڑٕ</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G26" s="5">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Zaen te su wuchaan chu</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G27" s="4">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Technical spiritual definition of ihsan; verify meaning against original Arabic.</t>
+          <t xml:space="preserve">Owner supplied Romanized phrase exactly; Kashmiri-script spelling and precise clause alignment not supplied.</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مَشکوٗک مَعٲملہٕ — یِمَن ہُنٛد حَلٲل یا حَرٲم آسُن صاف چھُنہٕ</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G28" s="5">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">قَبِیلہٕ ہُنٛد وَفد</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G29" s="4">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1398,12 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">بَتہٕ ہُنٛد اَکھ لُقمہٕ / اَکھ نِوالہٕ</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G30" s="5">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خٲلِص نَصیٖحَت / اَخلٲصہٕ سۭتۍ مَشوَرٕ دِیُن</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G31" s="4">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reviewed religious term: نصیحت / exact phrasing is a new draft</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1500,12 +1500,12 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">لُکَن برونٛہہ بَیعَت کَرُن / وَفٲدٲری ہُنٛد عَہد کَرُن</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G32" s="5">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing Bukhari 18 owner-approved terminology: بیعت</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">اَہل نہٕ ٲسَن وٲلِس شَخصَس ذِمہٕدٲری سونٛپُن</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G33" s="4">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1602,12 +1602,12 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">وضو وِزِ کھورِ نہ چھلُن</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G34" s="5">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner spelling for feet: تَمہِ سٕندۍ کھور (hadith-pref-007)</t>
+          <t xml:space="preserve">Exact owner-provided Kashmiri correction 2026-10-28. Previous draft retained.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync Kashmiri Bukhari vocabulary owner review through item 30
* Record Bukhari vocabulary 21–30 acceptance and corrections for 23 and 30

* Document owner review of vocabulary items 21 to 30

* Record approved vocabulary batch 21–30

* Update Bukhari review Excel with owner wording and acceptances through item 30
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -1143,12 +1143,12 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">فِسق — گُناہگارٕ عمل</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G25" s="4">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">دۄن شَخصَن دَرمِیان جَھگڑٕ</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G26" s="5">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Zaen te su wuchaan chu</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G27" s="4">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Technical spiritual definition of ihsan; verify meaning against original Arabic.</t>
+          <t xml:space="preserve">Owner supplied Romanized phrase exactly; Kashmiri-script spelling and precise clause alignment not supplied.</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مَشکوٗک مَعٲملہٕ — یِمَن ہُنٛد حَلٲل یا حَرٲم آسُن صاف چھُنہٕ</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G28" s="5">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">قَبِیلہٕ ہُنٛد وَفد</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G29" s="4">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1398,12 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">بَتہٕ ہُنٛد اَکھ لُقمہٕ / اَکھ نِوالہٕ</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G30" s="5">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1449,12 +1449,12 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خٲلِص نَصیٖحَت / اَخلٲصہٕ سۭتۍ مَشوَرٕ دِیُن</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G31" s="4">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reviewed religious term: نصیحت / exact phrasing is a new draft</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1500,12 +1500,12 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">لُکَن برونٛہہ بَیعَت کَرُن / وَفٲدٲری ہُنٛد عَہد کَرُن</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G32" s="5">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Existing Bukhari 18 owner-approved terminology: بیعت</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">اَہل نہٕ ٲسَن وٲلِس شَخصَس ذِمہٕدٲری سونٛپُن</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G33" s="4">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft phrase on 2026-10-28 (vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -1602,12 +1602,12 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">وضو وِزِ کھورِ نہ چھلُن</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G34" s="5">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner spelling for feet: تَمہِ سٕندۍ کھور (hadith-pref-007)</t>
+          <t xml:space="preserve">Exact owner-provided Kashmiri correction 2026-10-28. Previous draft retained.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Bukhari owner review Excel through item 40
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -1653,12 +1653,12 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Khazir kul</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G35" s="4">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1704,12 +1704,12 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">akh awoont kothean peath behith te برٛونٛہمہِ زنٛگہِ گٔنڈِتھ</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G36" s="5">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Camel equipment and exact verb need reviewer confirmation.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">صوٗبَک حٲکِم / والی</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G37" s="4">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1806,12 +1806,12 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مُہر وٲلۍ Waen</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G38" s="5">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مَجلِسَس منٛز بیٛاکِس شَخصَس جایہِ دِیُن</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G39" s="4">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Hurmaet wael cxour reath</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G40" s="5">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">baar baar waen parith lukh paraishan karen</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G41" s="4">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -2010,12 +2010,12 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خُشخَبٔری دِیُن</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G42" s="5">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -2061,12 +2061,12 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">دیٖنُک گٔہٕرٕ علم تہٕ سَمَجھ حٲصِل کَرُن</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G43" s="4">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -2112,12 +2112,12 @@
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Khazre khulech پوشن ہُند جھرمٹ</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G44" s="5">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rare botanical term; retain explanation until reviewed.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Save owner Kashmiri Hadith vocabulary review through item 40
* Record owner Kashmiri vocabulary corrections for 31 to 40

* Update Bukhari vocabulary review CSV for items 31-40

* Document owner review of Bukhari Kashmiri vocabulary 31-40

* Update Bukhari owner review Excel through item 40
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -1653,12 +1653,12 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Khazir kul</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G35" s="4">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1704,12 +1704,12 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">akh awoont kothean peath behith te برٛونٛہمہِ زنٛگہِ گٔنڈِتھ</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G36" s="5">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Camel equipment and exact verb need reviewer confirmation.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">صوٗبَک حٲکِم / والی</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G37" s="4">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1806,12 +1806,12 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مُہر وٲلۍ Waen</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G38" s="5">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مَجلِسَس منٛز بیٛاکِس شَخصَس جایہِ دِیُن</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G39" s="4">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Hurmaet wael cxour reath</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G40" s="5">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">baar baar waen parith lukh paraishan karen</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G41" s="4">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -2010,12 +2010,12 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خُشخَبٔری دِیُن</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G42" s="5">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -2061,12 +2061,12 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">دیٖنُک گٔہٕرٕ علم تہٕ سَمَجھ حٲصِل کَرُن</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G43" s="4">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>
@@ -2112,12 +2112,12 @@
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Khazre khulech پوشن ہُند جھرمٹ</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G44" s="5">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rare botanical term; retain explanation until reviewed.</t>
+          <t xml:space="preserve">Owner reviewed 2026-10-28. Original AI draft remains in column I.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync Bukhari Kashmiri review Excel with owner corrections 41–50
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -2163,12 +2163,12 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مٲل اللہ تعالہ سٕندِ وَتہِ منٛز دُرُست طَرٖیقَس پؠٹھ خَرچ کَرُن</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G45" s="4">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2214,12 +2214,12 @@
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">حضرت خَضِر علیہ السلام — حضرت موٗسیٰ علیہ السلامَن ہُنٛد ساتھی</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G46" s="5">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2265,12 +2265,12 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">بٲلِغ سَپدُن / بٔڈ عُمرَس واتُن</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G47" s="4">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2316,12 +2316,12 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">kear mnx balti seet aab kadun</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G48" s="5">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner provided 'kear' for well and the full Romanized expression; spelling in Kashmiri script is unconfirmed. Old AI draft preserved in I.</t>
         </is>
       </c>
     </row>
@@ -2367,12 +2367,12 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">حضرت موٗسیٰ علیہ السلامَن حضرت خَضِر علیہ السلام سۭتۍ مُلٲقات</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G49" s="4">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2418,12 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">زَرخؠز زٔمیٖن، یۄس روٗدُک آب پَنَس منٛز جذب کَران چھےٚ</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G50" s="5">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rainfall parable; check the soil terminology.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2469,12 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">بانٛج زٔمیٖن، یۄس روٗدُک آب نہٕ رَٹِ</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G51" s="4">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rainfall parable; check the soil terminology.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2520,12 +2520,12 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">قِیٲمَتَچ نِشٲنؠ / عَلامَتھ</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G52" s="5">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خوابُک تَعبیٖر کَرُن</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G53" s="4">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2622,12 +2622,12 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Quraabnei bronuh kaluk maees cxatun.</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G54" s="5">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Exact Romanized correction from owner for shaving the head before sacrifice; script spelling unconfirmed. Old AI draft preserved in I.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync owner-corrected Bukhari vocabulary through item 50
* Record owner corrections for well and head-shaving, vocabulary 41–50

* Record owner-review of Bukhari 41–50 terminology and corrections

* Document owner review for vocabulary 41–50

* Sync Bukhari Kashmiri review Excel with owner corrections 41–50
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -2163,12 +2163,12 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">مٲل اللہ تعالہ سٕندِ وَتہِ منٛز دُرُست طَرٖیقَس پؠٹھ خَرچ کَرُن</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G45" s="4">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2214,12 +2214,12 @@
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">حضرت خَضِر علیہ السلام — حضرت موٗسیٰ علیہ السلامَن ہُنٛد ساتھی</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G46" s="5">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2265,12 +2265,12 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">بٲلِغ سَپدُن / بٔڈ عُمرَس واتُن</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G47" s="4">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2316,12 +2316,12 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">kear mnx balti seet aab kadun</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G48" s="5">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner provided 'kear' for well and the full Romanized expression; spelling in Kashmiri script is unconfirmed. Old AI draft preserved in I.</t>
         </is>
       </c>
     </row>
@@ -2367,12 +2367,12 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">حضرت موٗسیٰ علیہ السلامَن حضرت خَضِر علیہ السلام سۭتۍ مُلٲقات</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G49" s="4">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2418,12 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">زَرخؠز زٔمیٖن، یۄس روٗدُک آب پَنَس منٛز جذب کَران چھےٚ</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G50" s="5">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rainfall parable; check the soil terminology.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2469,12 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">بانٛج زٔمیٖن، یۄس روٗدُک آب نہٕ رَٹِ</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G51" s="4">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rainfall parable; check the soil terminology.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2520,12 +2520,12 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">قِیٲمَتَچ نِشٲنؠ / عَلامَتھ</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G52" s="5">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خوابُک تَعبیٖر کَرُن</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G53" s="4">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted the draft wording in the 41–50 review on 2026-10-28; vocabulary only, not full hadith.</t>
         </is>
       </c>
     </row>
@@ -2622,12 +2622,12 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Quraabnei bronuh kaluk maees cxatun.</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G54" s="5">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Exact Romanized correction from owner for shaving the head before sacrifice; script spelling unconfirmed. Old AI draft preserved in I.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Bukhari Excel vocabulary review through item 60
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -2673,12 +2673,12 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jumratas peath loket kaneii lagawaeoun hajjas doraan</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G55" s="4">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preserves ritual name رَمی and Jamrat</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner raw input: Jumratas peath loket kaneii (for stones ) lagawaeoun(for throwing) hajjas doraan (during hajj). Romanized Kashmir wording retained, explanations not treated as part of the translation. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -2724,12 +2724,12 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ہَرج — بٔڈ پَیمانَس پؠٹھ لُکَن ہُنٛد قَتل</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G56" s="5">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -2775,12 +2775,12 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">سِرِس گِرَہَن / aftabs gruhun</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G57" s="4">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Natural term for eclipse requires confirmation.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner explicitly replaced soraj grhun (سوٗرَج گِرَہَن) with 'aftabs gruhun'. Earlier alternate سِرِس گِرَہَن remains a draft, not a separately approved native term. Roman spelling unconfirmed. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -2826,12 +2826,12 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">عَبدُالقَیس قَبِیلٕ ہُنٛد وَفد</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G58" s="5">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -2877,12 +2877,12 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">رَضٲعَت — دودھ چھوٚنہٕ سۭتۍ بَنَن وول رِشتٕ</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G59" s="4">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legal concept of milk kinship must be reviewed carefully.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -2928,12 +2928,12 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">وارِ وارِ کلاسس منز گژھُن</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G60" s="5">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied Perso-Arabic spelling preserved exactly. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2979,12 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jamaatech niamaaz wariya zeanth vannawaoyn</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G61" s="4">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied Romanized Kashmiri wording preserved exactly. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">رٲومُت چیز تہٕ یہ کِتھٕ کٔنۍ  پرزناوُن</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G62" s="5">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied Perso-Arabic wording, including spacing, preserved exactly. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3081,12 +3081,12 @@
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Paen te leatherooo thealee</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G63" s="4">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm historical lost-property container terminology.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied mixed English/Romanized wording preserved exactly; exact Kashmiri script/terms for leather container not confirmed. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3132,12 +3132,12 @@
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">نَسَبَس مُتعلِق سَوال — کُس چھُ تَمہِ سُنٛد مول؟</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G64" s="5">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record owner-approved Bukhari vocabulary review through item 60
* Update Bukhari vocabulary 51–60 with owner corrections and approvals

* Record owner corrections for Bukhari vocabulary items 51–60

* Document owner Bukhari vocabulary review 51–60

* Update Bukhari Excel vocabulary review through item 60
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -2673,12 +2673,12 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jumratas peath loket kaneii lagawaeoun hajjas doraan</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G55" s="4">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preserves ritual name رَمی and Jamrat</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner raw input: Jumratas peath loket kaneii (for stones ) lagawaeoun(for throwing) hajjas doraan (during hajj). Romanized Kashmir wording retained, explanations not treated as part of the translation. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -2724,12 +2724,12 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ہَرج — بٔڈ پَیمانَس پؠٹھ لُکَن ہُنٛد قَتل</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G56" s="5">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -2775,12 +2775,12 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">سِرِس گِرَہَن / aftabs gruhun</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G57" s="4">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Natural term for eclipse requires confirmation.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner explicitly replaced soraj grhun (سوٗرَج گِرَہَن) with 'aftabs gruhun'. Earlier alternate سِرِس گِرَہَن remains a draft, not a separately approved native term. Roman spelling unconfirmed. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -2826,12 +2826,12 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">عَبدُالقَیس قَبِیلٕ ہُنٛد وَفد</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G58" s="5">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -2877,12 +2877,12 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">رَضٲعَت — دودھ چھوٚنہٕ سۭتۍ بَنَن وول رِشتٕ</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G59" s="4">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legal concept of milk kinship must be reviewed carefully.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>
@@ -2928,12 +2928,12 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">وارِ وارِ کلاسس منز گژھُن</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G60" s="5">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied Perso-Arabic spelling preserved exactly. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2979,12 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jamaatech niamaaz wariya zeanth vannawaoyn</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G61" s="4">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied Romanized Kashmiri wording preserved exactly. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">رٲومُت چیز تہٕ یہ کِتھٕ کٔنۍ  پرزناوُن</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner corrected</t>
         </is>
       </c>
       <c r="G62" s="5">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied Perso-Arabic wording, including spacing, preserved exactly. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3081,12 +3081,12 @@
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Paen te leatherooo thealee</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G63" s="4">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm historical lost-property container terminology.</t>
+          <t xml:space="preserve">Owner correction 2026-10-28. Owner-supplied mixed English/Romanized wording preserved exactly; exact Kashmiri script/terms for leather container not confirmed. Original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3132,12 +3132,12 @@
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">نَسَبَس مُتعلِق سَوال — کُس چھُ تَمہِ سُنٛد مول؟</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G64" s="5">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted previously proposed expression as correct in review of items 51–60 on 2026-10-28; vocabulary only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync final approved 66-entry Kashmiri vocabulary Excel review
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -3183,12 +3183,12 @@
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">دَروازَس پؠٹھ تٕرٛے لَٹہٕ اِجازَت پرژھن</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G65" s="4">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3234,12 +3234,12 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Aaesmanei kitaban hend manen waek</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G66" s="5">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maintain precise scriptural-group definition from source.</t>
+          <t xml:space="preserve">Owner provided Romanized Kashmiri phrase exactly on 2026-10-28. Kashmiri-script spelling not yet owner-confirmed; original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3285,12 +3285,12 @@
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خَیرٲتَس منٛز دِنہٕ آمٕژۍ کَنَن ہٕندۍ douuuer</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G67" s="4">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm native word for earrings.</t>
+          <t xml:space="preserve">Owner instructed to replace word for earrings with 'douuuer' (Roman letters). Remainder of expression is earlier AI draft and not separately confirmed. Original proposal retained in I.</t>
         </is>
       </c>
     </row>
@@ -3336,12 +3336,12 @@
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">روزِ قِیٲمَتَس منٛز شَفٲعَت</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G68" s="5">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retains established religious term شفاعت</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3387,12 +3387,12 @@
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">عِلم بَغٲر دِیٖنی فَتویٰ دِیُن</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G69" s="4">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retains established religious term فتویٰ</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3438,12 +3438,12 @@
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">لُکَن گُمراہ کَرُن / غَلَط وَتہِ کُن نِیُن</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G70" s="5">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize Excel review guide with 66 of 66 vocabulary approvals and corrections
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -42,7 +42,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">66 draft terms · Hadith 27–100 · Enter your wording in column E; original draft in column I</t>
+          <t xml:space="preserve">Vocabulary review complete: 66 / 66 expressions · 39 accepted · 27 corrected · Complete Hadith narrations NOT yet approved</t>
         </is>
       </c>
     </row>
@@ -3543,28 +3543,28 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPORTANT: these are draft vocabulary proposals, NOT complete hadith translations.</t>
+          <t xml:space="preserve">FINAL REVIEW COMPLETE: 66 / 66 selected vocabulary expressions reviewed, NOT whole hadith narrations.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">They are NOT owner-approved; previous Cipher-reviewed wording remains untouched.</t>
+          <t xml:space="preserve">39 accepted as drafted; 27 corrected. Some Romanized owner corrections still need script confirmation.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The original proposed wording is preserved for comparison.</t>
+          <t xml:space="preserve">Column E contains owner wording; column F review status; column I retains original AI drafts.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOW confidence rows deserve extra attention.</t>
+          <t xml:space="preserve">Original AI confidence scores describe the draft, not the owner's approved wording.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete owner Kashmiri vocabulary review of all 66 Bukhari expressions
* Finish Kashmiri Bukhari vocabulary review for items 61-66

* Complete owner vocabulary correction ledger for 66 Sahih al-Bukhari expressions

* Document final approved vocabulary review and complete 66 item checklist

* Sync final approved 66-entry Kashmiri vocabulary Excel review

* Finalize Excel review guide with 66 of 66 vocabulary approvals and corrections

* Update Bukhari review documentation to distinguish completed vocabulary from unreviewed full hadiths
</commit_message>
<xml_diff>
--- a/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
+++ b/review-output/Bukhari_27-100_Kashmiri_Proposed_Translations.xlsx
@@ -42,7 +42,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">66 draft terms · Hadith 27–100 · Enter your wording in column E; original draft in column I</t>
+          <t xml:space="preserve">Vocabulary review complete: 66 / 66 expressions · 39 accepted · 27 corrected · Complete Hadith narrations NOT yet approved</t>
         </is>
       </c>
     </row>
@@ -3183,12 +3183,12 @@
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">دَروازَس پؠٹھ تٕرٛے لَٹہٕ اِجازَت پرژھن</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G65" s="4">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3234,12 +3234,12 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Aaesmanei kitaban hend manen waek</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G66" s="5">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maintain precise scriptural-group definition from source.</t>
+          <t xml:space="preserve">Owner provided Romanized Kashmiri phrase exactly on 2026-10-28. Kashmiri-script spelling not yet owner-confirmed; original AI draft retained in column I.</t>
         </is>
       </c>
     </row>
@@ -3285,12 +3285,12 @@
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">خَیرٲتَس منٛز دِنہٕ آمٕژۍ کَنَن ہٕندۍ douuuer</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner wording — script to confirm</t>
         </is>
       </c>
       <c r="G67" s="4">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm native word for earrings.</t>
+          <t xml:space="preserve">Owner instructed to replace word for earrings with 'douuuer' (Roman letters). Remainder of expression is earlier AI draft and not separately confirmed. Original proposal retained in I.</t>
         </is>
       </c>
     </row>
@@ -3336,12 +3336,12 @@
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">روزِ قِیٲمَتَس منٛز شَفٲعَت</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G68" s="5">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retains established religious term شفاعت</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3387,12 +3387,12 @@
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">عِلم بَغٲر دِیٖنی فَتویٰ دِیُن</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G69" s="4">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retains established religious term فتویٰ</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3438,12 +3438,12 @@
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">لُکَن گُمراہ کَرُن / غَلَط وَتہِ کُن نِیُن</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs review</t>
+          <t xml:space="preserve">Owner accepted</t>
         </is>
       </c>
       <c r="G70" s="5">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed wording from Cipher approved style and general Kashmiri usage; NOT owner-approved.</t>
+          <t xml:space="preserve">Owner accepted draft expression on 2026-10-28; vocabulary only, not full narration.</t>
         </is>
       </c>
     </row>
@@ -3543,28 +3543,28 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPORTANT: these are draft vocabulary proposals, NOT complete hadith translations.</t>
+          <t xml:space="preserve">FINAL REVIEW COMPLETE: 66 / 66 selected vocabulary expressions reviewed, NOT whole hadith narrations.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">They are NOT owner-approved; previous Cipher-reviewed wording remains untouched.</t>
+          <t xml:space="preserve">39 accepted as drafted; 27 corrected. Some Romanized owner corrections still need script confirmation.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The original proposed wording is preserved for comparison.</t>
+          <t xml:space="preserve">Column E contains owner wording; column F review status; column I retains original AI drafts.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOW confidence rows deserve extra attention.</t>
+          <t xml:space="preserve">Original AI confidence scores describe the draft, not the owner's approved wording.</t>
         </is>
       </c>
     </row>

</xml_diff>